<commit_message>
reworked player list definition
</commit_message>
<xml_diff>
--- a/S16/_members (2025).xlsx
+++ b/S16/_members (2025).xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="272" uniqueCount="267">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="271" uniqueCount="266">
   <si>
     <t xml:space="preserve">Role</t>
   </si>
@@ -818,18 +818,16 @@
   </si>
   <si>
     <t xml:space="preserve">kw1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1234</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="General"/>
-    <numFmt numFmtId="165" formatCode="000000"/>
+    <numFmt numFmtId="165" formatCode="0"/>
+    <numFmt numFmtId="166" formatCode="000000"/>
   </numFmts>
   <fonts count="7">
     <font>
@@ -931,7 +929,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -943,7 +941,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1146,7 +1144,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:V87"/>
+  <dimension ref="A1:X87"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="9.1"/>
@@ -1160,6 +1158,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="1" width="17.7"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="1" width="23.61"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="22" min="22" style="1" width="21.44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="24" min="24" style="2" width="9.91"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1208,8 +1207,9 @@
         <v>11</v>
       </c>
       <c r="D2" s="4"/>
-      <c r="E2" s="5" t="n">
-        <v>802975.382472669</v>
+      <c r="E2" s="5" t="str">
+        <f aca="true">TEXT(TRUNC(1000000*RAND()),"000000")</f>
+        <v>188959</v>
       </c>
       <c r="F2" s="6"/>
       <c r="G2" s="1" t="s">
@@ -1268,8 +1268,9 @@
         <v>21</v>
       </c>
       <c r="D3" s="4"/>
-      <c r="E3" s="5" t="n">
-        <v>955804.340271945</v>
+      <c r="E3" s="5" t="str">
+        <f aca="true">TEXT(TRUNC(1000000*RAND()),"000000")</f>
+        <v>655324</v>
       </c>
       <c r="G3" s="1" t="s">
         <v>22</v>
@@ -1336,8 +1337,9 @@
         <v>33</v>
       </c>
       <c r="D4" s="4"/>
-      <c r="E4" s="5" t="n">
-        <v>451266.054962523</v>
+      <c r="E4" s="5" t="str">
+        <f aca="true">TEXT(TRUNC(1000000*RAND()),"000000")</f>
+        <v>353303</v>
       </c>
       <c r="G4" s="1" t="s">
         <v>34</v>
@@ -1398,8 +1400,9 @@
         <v>43</v>
       </c>
       <c r="D5" s="4"/>
-      <c r="E5" s="5" t="n">
-        <v>109882.570337404</v>
+      <c r="E5" s="5" t="str">
+        <f aca="true">TEXT(TRUNC(1000000*RAND()),"000000")</f>
+        <v>816690</v>
       </c>
       <c r="G5" s="1" t="s">
         <v>44</v>
@@ -1442,8 +1445,9 @@
         <v>47</v>
       </c>
       <c r="D6" s="4"/>
-      <c r="E6" s="5" t="n">
-        <v>763478.933231578</v>
+      <c r="E6" s="5" t="str">
+        <f aca="true">TEXT(TRUNC(1000000*RAND()),"000000")</f>
+        <v>272599</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="13.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1457,8 +1461,9 @@
         <v>48</v>
       </c>
       <c r="D7" s="4"/>
-      <c r="E7" s="5" t="n">
-        <v>906569.401452616</v>
+      <c r="E7" s="5" t="str">
+        <f aca="true">TEXT(TRUNC(1000000*RAND()),"000000")</f>
+        <v>349816</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="13.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1472,8 +1477,9 @@
         <v>49</v>
       </c>
       <c r="D8" s="4"/>
-      <c r="E8" s="5" t="n">
-        <v>566668.857114141</v>
+      <c r="E8" s="5" t="str">
+        <f aca="true">TEXT(TRUNC(1000000*RAND()),"000000")</f>
+        <v>468157</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="13.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1487,8 +1493,9 @@
         <v>50</v>
       </c>
       <c r="D9" s="4"/>
-      <c r="E9" s="5" t="n">
-        <v>651067.140213711</v>
+      <c r="E9" s="5" t="str">
+        <f aca="true">TEXT(TRUNC(1000000*RAND()),"000000")</f>
+        <v>559637</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="13.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1502,8 +1509,9 @@
         <v>51</v>
       </c>
       <c r="D10" s="4"/>
-      <c r="E10" s="5" t="n">
-        <v>552288.43721353</v>
+      <c r="E10" s="5" t="str">
+        <f aca="true">TEXT(TRUNC(1000000*RAND()),"000000")</f>
+        <v>905804</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="13.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1517,8 +1525,9 @@
         <v>52</v>
       </c>
       <c r="D11" s="4"/>
-      <c r="E11" s="5" t="n">
-        <v>480759.091918243</v>
+      <c r="E11" s="5" t="str">
+        <f aca="true">TEXT(TRUNC(1000000*RAND()),"000000")</f>
+        <v>777792</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="13.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1532,8 +1541,9 @@
         <v>53</v>
       </c>
       <c r="D12" s="4"/>
-      <c r="E12" s="5" t="n">
-        <v>443248.589904883</v>
+      <c r="E12" s="5" t="str">
+        <f aca="true">TEXT(TRUNC(1000000*RAND()),"000000")</f>
+        <v>630032</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="13.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1547,8 +1557,9 @@
         <v>54</v>
       </c>
       <c r="D13" s="4"/>
-      <c r="E13" s="5" t="n">
-        <v>529144.653443627</v>
+      <c r="E13" s="5" t="str">
+        <f aca="true">TEXT(TRUNC(1000000*RAND()),"000000")</f>
+        <v>423437</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="13.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1562,8 +1573,9 @@
         <v>55</v>
       </c>
       <c r="D14" s="4"/>
-      <c r="E14" s="5" t="n">
-        <v>396204.92285183</v>
+      <c r="E14" s="5" t="str">
+        <f aca="true">TEXT(TRUNC(1000000*RAND()),"000000")</f>
+        <v>151747</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="13.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1575,8 +1587,9 @@
       </c>
       <c r="C15" s="4"/>
       <c r="D15" s="4"/>
-      <c r="E15" s="5" t="n">
-        <v>623257.192414307</v>
+      <c r="E15" s="5" t="str">
+        <f aca="true">TEXT(TRUNC(1000000*RAND()),"000000")</f>
+        <v>997609</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="13.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1590,8 +1603,9 @@
         <v>56</v>
       </c>
       <c r="D16" s="4"/>
-      <c r="E16" s="5" t="n">
-        <v>70214.7008728433</v>
+      <c r="E16" s="5" t="str">
+        <f aca="true">TEXT(TRUNC(1000000*RAND()),"000000")</f>
+        <v>934181</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="13.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1603,8 +1617,9 @@
       </c>
       <c r="C17" s="4"/>
       <c r="D17" s="4"/>
-      <c r="E17" s="5" t="n">
-        <v>747630.491661396</v>
+      <c r="E17" s="5" t="str">
+        <f aca="true">TEXT(TRUNC(1000000*RAND()),"000000")</f>
+        <v>819400</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="13.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1616,8 +1631,9 @@
       </c>
       <c r="C18" s="4"/>
       <c r="D18" s="4"/>
-      <c r="E18" s="5" t="n">
-        <v>824648.506272575</v>
+      <c r="E18" s="5" t="str">
+        <f aca="true">TEXT(TRUNC(1000000*RAND()),"000000")</f>
+        <v>609941</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="13.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1631,8 +1647,9 @@
         <v>57</v>
       </c>
       <c r="D19" s="4"/>
-      <c r="E19" s="5" t="n">
-        <v>49595.1579423887</v>
+      <c r="E19" s="5" t="str">
+        <f aca="true">TEXT(TRUNC(1000000*RAND()),"000000")</f>
+        <v>620573</v>
       </c>
       <c r="G19" s="1" t="s">
         <v>58</v>
@@ -1693,8 +1710,9 @@
         <v>67</v>
       </c>
       <c r="D20" s="4"/>
-      <c r="E20" s="5" t="n">
-        <v>751644.292809301</v>
+      <c r="E20" s="5" t="str">
+        <f aca="true">TEXT(TRUNC(1000000*RAND()),"000000")</f>
+        <v>391500</v>
       </c>
       <c r="G20" s="1" t="s">
         <v>68</v>
@@ -1755,8 +1773,9 @@
         <v>77</v>
       </c>
       <c r="D21" s="4"/>
-      <c r="E21" s="5" t="n">
-        <v>242150.486357673</v>
+      <c r="E21" s="5" t="str">
+        <f aca="true">TEXT(TRUNC(1000000*RAND()),"000000")</f>
+        <v>239647</v>
       </c>
       <c r="G21" s="1" t="s">
         <v>78</v>
@@ -1823,8 +1842,9 @@
         <v>89</v>
       </c>
       <c r="D22" s="4"/>
-      <c r="E22" s="5" t="n">
-        <v>282296.297065066</v>
+      <c r="E22" s="5" t="str">
+        <f aca="true">TEXT(TRUNC(1000000*RAND()),"000000")</f>
+        <v>845596</v>
       </c>
       <c r="G22" s="1" t="s">
         <v>90</v>
@@ -1891,8 +1911,9 @@
         <v>101</v>
       </c>
       <c r="D23" s="4"/>
-      <c r="E23" s="5" t="n">
-        <v>208153.700721655</v>
+      <c r="E23" s="5" t="str">
+        <f aca="true">TEXT(TRUNC(1000000*RAND()),"000000")</f>
+        <v>034934</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="13.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1906,8 +1927,9 @@
         <v>102</v>
       </c>
       <c r="D24" s="4"/>
-      <c r="E24" s="5" t="n">
-        <v>418063.696147085</v>
+      <c r="E24" s="5" t="str">
+        <f aca="true">TEXT(TRUNC(1000000*RAND()),"000000")</f>
+        <v>972499</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="13.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1921,8 +1943,9 @@
         <v>103</v>
       </c>
       <c r="D25" s="4"/>
-      <c r="E25" s="5" t="n">
-        <v>450145.89410187</v>
+      <c r="E25" s="5" t="str">
+        <f aca="true">TEXT(TRUNC(1000000*RAND()),"000000")</f>
+        <v>304980</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="13.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1936,8 +1959,9 @@
         <v>104</v>
       </c>
       <c r="D26" s="4"/>
-      <c r="E26" s="5" t="n">
-        <v>567181.277705738</v>
+      <c r="E26" s="5" t="str">
+        <f aca="true">TEXT(TRUNC(1000000*RAND()),"000000")</f>
+        <v>400903</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="13.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1951,8 +1975,9 @@
         <v>105</v>
       </c>
       <c r="D27" s="4"/>
-      <c r="E27" s="5" t="n">
-        <v>20643.5329397866</v>
+      <c r="E27" s="5" t="str">
+        <f aca="true">TEXT(TRUNC(1000000*RAND()),"000000")</f>
+        <v>972466</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="13.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1966,8 +1991,9 @@
         <v>106</v>
       </c>
       <c r="D28" s="4"/>
-      <c r="E28" s="5" t="n">
-        <v>795108.603499209</v>
+      <c r="E28" s="5" t="str">
+        <f aca="true">TEXT(TRUNC(1000000*RAND()),"000000")</f>
+        <v>223759</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="13.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1981,8 +2007,9 @@
         <v>107</v>
       </c>
       <c r="D29" s="4"/>
-      <c r="E29" s="5" t="n">
-        <v>375.149369804374</v>
+      <c r="E29" s="5" t="str">
+        <f aca="true">TEXT(TRUNC(1000000*RAND()),"000000")</f>
+        <v>825900</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="13.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1996,8 +2023,9 @@
         <v>108</v>
       </c>
       <c r="D30" s="4"/>
-      <c r="E30" s="5" t="n">
-        <v>769954.391940447</v>
+      <c r="E30" s="5" t="str">
+        <f aca="true">TEXT(TRUNC(1000000*RAND()),"000000")</f>
+        <v>960107</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="13.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2011,8 +2039,9 @@
         <v>109</v>
       </c>
       <c r="D31" s="4"/>
-      <c r="E31" s="5" t="n">
-        <v>943228.120514321</v>
+      <c r="E31" s="5" t="str">
+        <f aca="true">TEXT(TRUNC(1000000*RAND()),"000000")</f>
+        <v>501357</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="13.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2026,8 +2055,9 @@
         <v>110</v>
       </c>
       <c r="D32" s="4"/>
-      <c r="E32" s="5" t="n">
-        <v>777529.235122408</v>
+      <c r="E32" s="5" t="str">
+        <f aca="true">TEXT(TRUNC(1000000*RAND()),"000000")</f>
+        <v>006813</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="13.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2041,8 +2071,9 @@
         <v>111</v>
       </c>
       <c r="D33" s="4"/>
-      <c r="E33" s="5" t="n">
-        <v>177645.896116461</v>
+      <c r="E33" s="5" t="str">
+        <f aca="true">TEXT(TRUNC(1000000*RAND()),"000000")</f>
+        <v>624293</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="13.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2056,8 +2087,9 @@
         <v>112</v>
       </c>
       <c r="D34" s="4"/>
-      <c r="E34" s="5" t="n">
-        <v>701186.64630769</v>
+      <c r="E34" s="5" t="str">
+        <f aca="true">TEXT(TRUNC(1000000*RAND()),"000000")</f>
+        <v>385048</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="13.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2071,8 +2103,9 @@
         <v>113</v>
       </c>
       <c r="D35" s="4"/>
-      <c r="E35" s="5" t="n">
-        <v>891708.123411197</v>
+      <c r="E35" s="5" t="str">
+        <f aca="true">TEXT(TRUNC(1000000*RAND()),"000000")</f>
+        <v>784873</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="13.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2086,8 +2119,9 @@
         <v>114</v>
       </c>
       <c r="D36" s="4"/>
-      <c r="E36" s="5" t="n">
-        <v>480954.383269504</v>
+      <c r="E36" s="5" t="str">
+        <f aca="true">TEXT(TRUNC(1000000*RAND()),"000000")</f>
+        <v>334840</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="13.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2101,8 +2135,9 @@
         <v>115</v>
       </c>
       <c r="D37" s="4"/>
-      <c r="E37" s="5" t="n">
-        <v>226310.349139848</v>
+      <c r="E37" s="5" t="str">
+        <f aca="true">TEXT(TRUNC(1000000*RAND()),"000000")</f>
+        <v>170869</v>
       </c>
       <c r="G37" s="1" t="s">
         <v>116</v>
@@ -2163,8 +2198,9 @@
         <v>125</v>
       </c>
       <c r="D38" s="4"/>
-      <c r="E38" s="5" t="n">
-        <v>979154.180225223</v>
+      <c r="E38" s="5" t="str">
+        <f aca="true">TEXT(TRUNC(1000000*RAND()),"000000")</f>
+        <v>512560</v>
       </c>
       <c r="G38" s="1" t="s">
         <v>126</v>
@@ -2225,8 +2261,9 @@
         <v>135</v>
       </c>
       <c r="D39" s="4"/>
-      <c r="E39" s="5" t="n">
-        <v>529864.263429908</v>
+      <c r="E39" s="5" t="str">
+        <f aca="true">TEXT(TRUNC(1000000*RAND()),"000000")</f>
+        <v>594776</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="13.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2240,8 +2277,9 @@
         <v>136</v>
       </c>
       <c r="D40" s="4"/>
-      <c r="E40" s="5" t="n">
-        <v>764917.043199876</v>
+      <c r="E40" s="5" t="str">
+        <f aca="true">TEXT(TRUNC(1000000*RAND()),"000000")</f>
+        <v>474082</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="13.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2255,8 +2293,9 @@
         <v>137</v>
       </c>
       <c r="D41" s="4"/>
-      <c r="E41" s="5" t="n">
-        <v>369815.377425931</v>
+      <c r="E41" s="5" t="str">
+        <f aca="true">TEXT(TRUNC(1000000*RAND()),"000000")</f>
+        <v>908060</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="13.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2270,8 +2309,9 @@
         <v>138</v>
       </c>
       <c r="D42" s="4"/>
-      <c r="E42" s="5" t="n">
-        <v>852660.599435625</v>
+      <c r="E42" s="5" t="str">
+        <f aca="true">TEXT(TRUNC(1000000*RAND()),"000000")</f>
+        <v>349851</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="13.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2285,8 +2325,9 @@
         <v>139</v>
       </c>
       <c r="D43" s="4"/>
-      <c r="E43" s="5" t="n">
-        <v>444097.164228061</v>
+      <c r="E43" s="5" t="str">
+        <f aca="true">TEXT(TRUNC(1000000*RAND()),"000000")</f>
+        <v>283207</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="13.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2300,8 +2341,9 @@
         <v>140</v>
       </c>
       <c r="D44" s="4"/>
-      <c r="E44" s="5" t="n">
-        <v>276626.702724514</v>
+      <c r="E44" s="5" t="str">
+        <f aca="true">TEXT(TRUNC(1000000*RAND()),"000000")</f>
+        <v>379779</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="13.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2315,8 +2357,9 @@
         <v>141</v>
       </c>
       <c r="D45" s="4"/>
-      <c r="E45" s="5" t="n">
-        <v>508877.055390987</v>
+      <c r="E45" s="5" t="str">
+        <f aca="true">TEXT(TRUNC(1000000*RAND()),"000000")</f>
+        <v>936340</v>
       </c>
       <c r="G45" s="1" t="s">
         <v>142</v>
@@ -2383,8 +2426,9 @@
         <v>153</v>
       </c>
       <c r="D46" s="4"/>
-      <c r="E46" s="5" t="n">
-        <v>60111.2233924169</v>
+      <c r="E46" s="5" t="str">
+        <f aca="true">TEXT(TRUNC(1000000*RAND()),"000000")</f>
+        <v>297603</v>
       </c>
       <c r="G46" s="1" t="s">
         <v>154</v>
@@ -2445,8 +2489,9 @@
         <v>163</v>
       </c>
       <c r="D47" s="4"/>
-      <c r="E47" s="5" t="n">
-        <v>864386.426764805</v>
+      <c r="E47" s="5" t="str">
+        <f aca="true">TEXT(TRUNC(1000000*RAND()),"000000")</f>
+        <v>995804</v>
       </c>
       <c r="G47" s="1" t="s">
         <v>164</v>
@@ -2501,8 +2546,9 @@
         <v>171</v>
       </c>
       <c r="D48" s="4"/>
-      <c r="E48" s="5" t="n">
-        <v>511308.837090815</v>
+      <c r="E48" s="5" t="str">
+        <f aca="true">TEXT(TRUNC(1000000*RAND()),"000000")</f>
+        <v>835781</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="13.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2516,8 +2562,9 @@
         <v>172</v>
       </c>
       <c r="D49" s="4"/>
-      <c r="E49" s="5" t="n">
-        <v>908521.789913416</v>
+      <c r="E49" s="5" t="str">
+        <f aca="true">TEXT(TRUNC(1000000*RAND()),"000000")</f>
+        <v>554333</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="13.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2531,8 +2578,9 @@
         <v>173</v>
       </c>
       <c r="D50" s="4"/>
-      <c r="E50" s="5" t="n">
-        <v>65609.3982717915</v>
+      <c r="E50" s="5" t="str">
+        <f aca="true">TEXT(TRUNC(1000000*RAND()),"000000")</f>
+        <v>627857</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="13.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2546,8 +2594,9 @@
         <v>174</v>
       </c>
       <c r="D51" s="4"/>
-      <c r="E51" s="5" t="n">
-        <v>267500.343391047</v>
+      <c r="E51" s="5" t="str">
+        <f aca="true">TEXT(TRUNC(1000000*RAND()),"000000")</f>
+        <v>460716</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="13.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2561,8 +2610,9 @@
         <v>175</v>
       </c>
       <c r="D52" s="4"/>
-      <c r="E52" s="5" t="n">
-        <v>699415.279626662</v>
+      <c r="E52" s="5" t="str">
+        <f aca="true">TEXT(TRUNC(1000000*RAND()),"000000")</f>
+        <v>858717</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="13.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2576,8 +2626,9 @@
         <v>176</v>
       </c>
       <c r="D53" s="4"/>
-      <c r="E53" s="5" t="n">
-        <v>484289.550587555</v>
+      <c r="E53" s="5" t="str">
+        <f aca="true">TEXT(TRUNC(1000000*RAND()),"000000")</f>
+        <v>308822</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="13.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2591,8 +2642,9 @@
         <v>177</v>
       </c>
       <c r="D54" s="4"/>
-      <c r="E54" s="5" t="n">
-        <v>690657.565270717</v>
+      <c r="E54" s="5" t="str">
+        <f aca="true">TEXT(TRUNC(1000000*RAND()),"000000")</f>
+        <v>458045</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="13.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2606,8 +2658,9 @@
         <v>178</v>
       </c>
       <c r="D55" s="4"/>
-      <c r="E55" s="5" t="n">
-        <v>944194.729283117</v>
+      <c r="E55" s="5" t="str">
+        <f aca="true">TEXT(TRUNC(1000000*RAND()),"000000")</f>
+        <v>988083</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="13.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2621,8 +2674,9 @@
         <v>179</v>
       </c>
       <c r="D56" s="4"/>
-      <c r="E56" s="5" t="n">
-        <v>998612.691374319</v>
+      <c r="E56" s="5" t="str">
+        <f aca="true">TEXT(TRUNC(1000000*RAND()),"000000")</f>
+        <v>059110</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="13.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2636,8 +2690,9 @@
         <v>180</v>
       </c>
       <c r="D57" s="4"/>
-      <c r="E57" s="5" t="n">
-        <v>673727.394016001</v>
+      <c r="E57" s="5" t="str">
+        <f aca="true">TEXT(TRUNC(1000000*RAND()),"000000")</f>
+        <v>827351</v>
       </c>
       <c r="G57" s="1" t="s">
         <v>181</v>
@@ -2704,8 +2759,9 @@
         <v>191</v>
       </c>
       <c r="D58" s="4"/>
-      <c r="E58" s="5" t="n">
-        <v>742044.989433403</v>
+      <c r="E58" s="5" t="str">
+        <f aca="true">TEXT(TRUNC(1000000*RAND()),"000000")</f>
+        <v>140797</v>
       </c>
       <c r="G58" s="1" t="s">
         <v>192</v>
@@ -2766,8 +2822,9 @@
         <v>201</v>
       </c>
       <c r="D59" s="4"/>
-      <c r="E59" s="5" t="n">
-        <v>652440.014717802</v>
+      <c r="E59" s="5" t="str">
+        <f aca="true">TEXT(TRUNC(1000000*RAND()),"000000")</f>
+        <v>496717</v>
       </c>
       <c r="G59" s="1" t="s">
         <v>202</v>
@@ -2828,8 +2885,9 @@
         <v>211</v>
       </c>
       <c r="D60" s="4"/>
-      <c r="E60" s="5" t="n">
-        <v>391176.7701218</v>
+      <c r="E60" s="5" t="str">
+        <f aca="true">TEXT(TRUNC(1000000*RAND()),"000000")</f>
+        <v>330545</v>
       </c>
       <c r="J60" s="3"/>
       <c r="M60" s="3"/>
@@ -2848,8 +2906,9 @@
         <v>212</v>
       </c>
       <c r="D61" s="4"/>
-      <c r="E61" s="5" t="n">
-        <v>976507.674873555</v>
+      <c r="E61" s="5" t="str">
+        <f aca="true">TEXT(TRUNC(1000000*RAND()),"000000")</f>
+        <v>494940</v>
       </c>
       <c r="J61" s="3"/>
       <c r="M61" s="3"/>
@@ -2868,8 +2927,9 @@
         <v>213</v>
       </c>
       <c r="D62" s="4"/>
-      <c r="E62" s="5" t="n">
-        <v>896812.103679734</v>
+      <c r="E62" s="5" t="str">
+        <f aca="true">TEXT(TRUNC(1000000*RAND()),"000000")</f>
+        <v>515661</v>
       </c>
       <c r="G62" s="1" t="s">
         <v>214</v>
@@ -2930,8 +2990,9 @@
         <v>223</v>
       </c>
       <c r="D63" s="4"/>
-      <c r="E63" s="5" t="n">
-        <v>552485.88315331</v>
+      <c r="E63" s="5" t="str">
+        <f aca="true">TEXT(TRUNC(1000000*RAND()),"000000")</f>
+        <v>179679</v>
       </c>
       <c r="G63" s="1" t="s">
         <v>224</v>
@@ -2992,8 +3053,9 @@
         <v>233</v>
       </c>
       <c r="D64" s="4"/>
-      <c r="E64" s="5" t="n">
-        <v>964142.781285241</v>
+      <c r="E64" s="5" t="str">
+        <f aca="true">TEXT(TRUNC(1000000*RAND()),"000000")</f>
+        <v>789129</v>
       </c>
       <c r="G64" s="1" t="s">
         <v>234</v>
@@ -3054,8 +3116,9 @@
         <v>243</v>
       </c>
       <c r="D65" s="4"/>
-      <c r="E65" s="5" t="n">
-        <v>689820.370694902</v>
+      <c r="E65" s="5" t="str">
+        <f aca="true">TEXT(TRUNC(1000000*RAND()),"000000")</f>
+        <v>226842</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="13.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3069,8 +3132,9 @@
         <v>244</v>
       </c>
       <c r="D66" s="4"/>
-      <c r="E66" s="5" t="n">
-        <v>528295.666754772</v>
+      <c r="E66" s="5" t="str">
+        <f aca="true">TEXT(TRUNC(1000000*RAND()),"000000")</f>
+        <v>368942</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="13.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3084,8 +3148,9 @@
         <v>245</v>
       </c>
       <c r="D67" s="4"/>
-      <c r="E67" s="5" t="n">
-        <v>831643.321075099</v>
+      <c r="E67" s="5" t="str">
+        <f aca="true">TEXT(TRUNC(1000000*RAND()),"000000")</f>
+        <v>065167</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="13.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3099,8 +3164,9 @@
         <v>246</v>
       </c>
       <c r="D68" s="4"/>
-      <c r="E68" s="5" t="n">
-        <v>289095.042185713</v>
+      <c r="E68" s="5" t="str">
+        <f aca="true">TEXT(TRUNC(1000000*RAND()),"000000")</f>
+        <v>507968</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="13.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3114,8 +3180,9 @@
         <v>247</v>
       </c>
       <c r="D69" s="4"/>
-      <c r="E69" s="5" t="n">
-        <v>982418.28793374</v>
+      <c r="E69" s="5" t="str">
+        <f aca="true">TEXT(TRUNC(1000000*RAND()),"000000")</f>
+        <v>309641</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="13.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3129,8 +3196,9 @@
         <v>248</v>
       </c>
       <c r="D70" s="4"/>
-      <c r="E70" s="5" t="n">
-        <v>157854.356062846</v>
+      <c r="E70" s="5" t="str">
+        <f aca="true">TEXT(TRUNC(1000000*RAND()),"000000")</f>
+        <v>987339</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="13.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3144,8 +3212,9 @@
         <v>249</v>
       </c>
       <c r="D71" s="4"/>
-      <c r="E71" s="5" t="n">
-        <v>100711.345256161</v>
+      <c r="E71" s="5" t="str">
+        <f aca="true">TEXT(TRUNC(1000000*RAND()),"000000")</f>
+        <v>963174</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="13.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3159,8 +3228,9 @@
         <v>250</v>
       </c>
       <c r="D72" s="4"/>
-      <c r="E72" s="5" t="n">
-        <v>199120.825125476</v>
+      <c r="E72" s="5" t="str">
+        <f aca="true">TEXT(TRUNC(1000000*RAND()),"000000")</f>
+        <v>964564</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="13.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3174,8 +3244,9 @@
         <v>251</v>
       </c>
       <c r="D73" s="4"/>
-      <c r="E73" s="5" t="n">
-        <v>966507.807841239</v>
+      <c r="E73" s="5" t="str">
+        <f aca="true">TEXT(TRUNC(1000000*RAND()),"000000")</f>
+        <v>908863</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="13.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3189,8 +3260,9 @@
         <v>252</v>
       </c>
       <c r="D74" s="4"/>
-      <c r="E74" s="5" t="n">
-        <v>335561.493258982</v>
+      <c r="E74" s="5" t="str">
+        <f aca="true">TEXT(TRUNC(1000000*RAND()),"000000")</f>
+        <v>760784</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="13.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3204,8 +3276,9 @@
         <v>253</v>
       </c>
       <c r="D75" s="4"/>
-      <c r="E75" s="5" t="n">
-        <v>240297.276805031</v>
+      <c r="E75" s="5" t="str">
+        <f aca="true">TEXT(TRUNC(1000000*RAND()),"000000")</f>
+        <v>962808</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="13.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3219,8 +3292,9 @@
         <v>254</v>
       </c>
       <c r="D76" s="7"/>
-      <c r="E76" s="5" t="n">
-        <v>338498.450176425</v>
+      <c r="E76" s="5" t="str">
+        <f aca="true">TEXT(TRUNC(1000000*RAND()),"000000")</f>
+        <v>502637</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="13.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3234,8 +3308,9 @@
         <v>255</v>
       </c>
       <c r="D77" s="7"/>
-      <c r="E77" s="5" t="n">
-        <v>981162.633471125</v>
+      <c r="E77" s="5" t="str">
+        <f aca="true">TEXT(TRUNC(1000000*RAND()),"000000")</f>
+        <v>746165</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="13.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3249,8 +3324,9 @@
         <v>256</v>
       </c>
       <c r="D78" s="4"/>
-      <c r="E78" s="5" t="n">
-        <v>851864.644099338</v>
+      <c r="E78" s="5" t="str">
+        <f aca="true">TEXT(TRUNC(1000000*RAND()),"000000")</f>
+        <v>557046</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="13.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3264,8 +3340,9 @@
         <v>257</v>
       </c>
       <c r="D79" s="4"/>
-      <c r="E79" s="5" t="n">
-        <v>726502.585934138</v>
+      <c r="E79" s="5" t="str">
+        <f aca="true">TEXT(TRUNC(1000000*RAND()),"000000")</f>
+        <v>669717</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="13.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3279,8 +3356,9 @@
         <v>258</v>
       </c>
       <c r="D80" s="4"/>
-      <c r="E80" s="5" t="n">
-        <v>142239.60245409</v>
+      <c r="E80" s="5" t="str">
+        <f aca="true">TEXT(TRUNC(1000000*RAND()),"000000")</f>
+        <v>258251</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="13.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3294,8 +3372,9 @@
         <v>259</v>
       </c>
       <c r="D81" s="4"/>
-      <c r="E81" s="5" t="n">
-        <v>730167.807828822</v>
+      <c r="E81" s="5" t="str">
+        <f aca="true">TEXT(TRUNC(1000000*RAND()),"000000")</f>
+        <v>029831</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="13.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3307,8 +3386,9 @@
       </c>
       <c r="C82" s="4"/>
       <c r="D82" s="4"/>
-      <c r="E82" s="5" t="n">
-        <v>585877.993141175</v>
+      <c r="E82" s="5" t="str">
+        <f aca="true">TEXT(TRUNC(1000000*RAND()),"000000")</f>
+        <v>908581</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="13.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3320,8 +3400,9 @@
       </c>
       <c r="C83" s="4"/>
       <c r="D83" s="4"/>
-      <c r="E83" s="5" t="n">
-        <v>965084.068471103</v>
+      <c r="E83" s="5" t="str">
+        <f aca="true">TEXT(TRUNC(1000000*RAND()),"000000")</f>
+        <v>992718</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="13.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3333,8 +3414,9 @@
       </c>
       <c r="C84" s="4"/>
       <c r="D84" s="4"/>
-      <c r="E84" s="5" t="n">
-        <v>512449.495355232</v>
+      <c r="E84" s="5" t="str">
+        <f aca="true">TEXT(TRUNC(1000000*RAND()),"000000")</f>
+        <v>588252</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3348,15 +3430,16 @@
         <v>261</v>
       </c>
       <c r="D85" s="1"/>
-      <c r="E85" s="5" t="n">
-        <v>761566.033490562</v>
+      <c r="E85" s="5" t="str">
+        <f aca="true">TEXT(TRUNC(1000000*RAND()),"000000")</f>
+        <v>209473</v>
       </c>
       <c r="F85" s="6" t="s">
         <v>262</v>
       </c>
-      <c r="G85" s="5" t="n">
-        <f aca="true">1000000*RAND()</f>
-        <v>272219.220023244</v>
+      <c r="G85" s="5" t="str">
+        <f aca="true">TEXT(TRUNC(1000000*RAND()),"000000")</f>
+        <v>856433</v>
       </c>
       <c r="H85" s="8" t="s">
         <v>263</v>
@@ -3372,12 +3455,14 @@
       <c r="C86" s="1" t="s">
         <v>265</v>
       </c>
-      <c r="E86" s="9" t="n">
-        <v>18123.5300141561</v>
+      <c r="E86" s="5" t="str">
+        <f aca="true">TEXT(TRUNC(1000000*RAND()),"000000")</f>
+        <v>866222</v>
       </c>
       <c r="F86" s="6" t="s">
         <v>265</v>
       </c>
+      <c r="X86" s="9"/>
     </row>
     <row r="87" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="1" t="s">
@@ -3389,8 +3474,9 @@
       <c r="C87" s="1" t="s">
         <v>261</v>
       </c>
-      <c r="E87" s="2" t="s">
-        <v>266</v>
+      <c r="E87" s="5" t="str">
+        <f aca="true">TEXT(TRUNC(1000000*RAND()),"000000")</f>
+        <v>379466</v>
       </c>
       <c r="F87" s="1" t="s">
         <v>261</v>

</xml_diff>